<commit_message>
Add README and enhance scraper to search multiple last names.
This update includes:
- A new `README.md` file with instructions on how to set up and run the scraper.
- Modification of the `scraper.py` script to iterate through a predefined list of common Latino last names.
- Aggregation of results from all searches into a single dataset before saving to output files.
- The output files (CSV, Excel, PDF) now contain the combined data from all searches.
</commit_message>
<xml_diff>
--- a/utah_county_data.xlsx
+++ b/utah_county_data.xlsx
@@ -1256,22 +1256,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GARCIA, ALICIA PAGE</t>
+          <t>RODRIGUEZ FAMILY TRUST 04-05-2023</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>607 N 1300 WEST</t>
+          <t>722 N 1130 WEST</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LEHI</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>84043</t>
+          <t>84057-3517</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1283,22 +1283,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GARCIA, ALIZON</t>
+          <t>RODRIGUEZ FAMILY TRUST 04-05-2023</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1397 W 1450 SOUTH</t>
+          <t>607 N 1660 WEST</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>LINDON</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>84663</t>
+          <t>84057-3517</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1310,22 +1310,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GARCIA, ALMA L GONZALEZ</t>
+          <t>RODRIGUEZ GARCI, ALIX</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>330 N 985 WEST</t>
+          <t>596 N LYNNBROOK DR</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>SPANISH FORK</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>84097</t>
+          <t>84660-1378</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1337,22 +1337,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GARCIA, ALONDRA JACKELINE</t>
+          <t>RODRIGUEZ PATINO, PLACIDO</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1355 W 1050 SOUTH</t>
+          <t>2304 E COYOTE ST</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>84663</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1364,22 +1364,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GARCIA, ALYSSA</t>
+          <t>RODRIGUEZ RENTAL EIGHT LLC</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>7049 N GOLDEN ACRES LOOP</t>
+          <t>655 S 50 WEST</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1391,22 +1391,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GARCIA, AMY</t>
+          <t>RODRIGUEZ RENTAL ONE LLC</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>5347 W WILLEM PL</t>
+          <t>45 W SMITH LN</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HIGHLAND</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>84003</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1418,12 +1418,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GARCIA, ANA KATYA SANCHEZ</t>
+          <t>RODRIGUEZ RENTAL SEVEN LLC</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>546 S 2150 WEST</t>
+          <t>675 S 50 WEST</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>84062</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1445,18 +1445,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GARCIA, ANA KATYA SANCHEZ</t>
+          <t>RODRIGUEZ RENTAL TWO LLC</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>540 S MAIN</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
           <t>PLEASANT GROVE</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>84062</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1468,22 +1472,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GARCIA, ANA MARIA</t>
+          <t>RODRIGUEZ, ABELARDO HIGUERA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>475 W 1890 SOUTH</t>
+          <t>2312 E WOODBURY LN</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PAYSON</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>84651</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1495,22 +1499,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GARCIA, ANDREA CHIGUIL</t>
+          <t>RODRIGUEZ, ADALBERTO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>628 W 1000 SOUTH</t>
+          <t>923 W 550 NORTH</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>84663</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1522,22 +1526,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GARCIA, ANDREINA D HERNANDEZ</t>
+          <t>RODRIGUEZ, ADALBERTO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>4877 S OLIVE AVE</t>
+          <t>490 S GENEVA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MAPLETON</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>84664</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1549,22 +1553,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GARCIA, ANDRES</t>
+          <t>RODRIGUEZ, ADALBERTO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2309 E 1650 SOUTH</t>
+          <t>50 W SMITH LN</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SPANISH FORK</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>84660</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1576,22 +1580,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GARCIA, ANDRES M</t>
+          <t>RODRIGUEZ, ADALBERTO</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>169 S 700 WEST</t>
+          <t>115 W HALE DR</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PROVO</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>84601-4251</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1603,22 +1607,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GARCIA, ANDRES M</t>
+          <t>RODRIGUEZ, ADALBERTO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>960 W 100 SOUTH</t>
+          <t>60 W HALE DR</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PROVO</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>84601-4003</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1630,22 +1634,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GARCIA, ANDREW M</t>
+          <t>RODRIGUEZ, ADALBERTO</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>3097 E SNOWY OWL CIR</t>
+          <t>630 S 50 WEST</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1657,22 +1661,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>GARCIA, ANEL L REYES</t>
+          <t>RODRIGUEZ, ADALBERTO</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2710 N 3720 WEST</t>
+          <t>690 S 50 WEST</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LEHI</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>84043</t>
+          <t>84062-2192</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1684,22 +1688,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GARCIA, ANGELA</t>
+          <t>RODRIGUEZ, ADAN MAGANA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>182 E 400 SOUTH</t>
+          <t>375 HARRISON AVE</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>GENOLA</t>
+          <t>AMERICAN FORK</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>84655</t>
+          <t>84003</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1711,22 +1715,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>GARCIA, ANGELA L</t>
+          <t>RODRIGUEZ, ADOLFO RODRIGUEZ</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>12925 W 14650 SOUTH</t>
+          <t>514 W 800 SOUTH</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ELBERTA</t>
+          <t>PAYSON</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>84626-0126</t>
+          <t>84651-2747</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1738,22 +1742,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GARCIA, ANN</t>
+          <t>RODRIGUEZ, ADRIAN</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1026 E 900 SOUTH</t>
+          <t>855 E 1330 SOUTH</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>SPANISH FORK</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>84663-2310</t>
+          <t>84660-2988</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1765,22 +1769,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>GARCIA, ANNETTE</t>
+          <t>RODRIGUEZ, ADRIAN GUSTAVO</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>930 S WOODLAND HILLS DR</t>
+          <t>6088 N SHEPS RIDGE RD</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>WOODLAND HILLS</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>84653-2063</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1792,22 +1796,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>GARCIA, ANTHONY</t>
+          <t>RODRIGUEZ, ADRIANA</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1397 W 1450 SOUTH</t>
+          <t>2043 S MOUNTAIN VISTA LN</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>84663</t>
+          <t>84606</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1819,22 +1823,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GARCIA, APOLONIO</t>
+          <t>RODRIGUEZ, AFRICA G</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1020 E 1200 SOUTH</t>
+          <t>265 N 800 WEST</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>SPANISH FORK</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>84663-2811</t>
+          <t>84660-3307</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -1846,12 +1850,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GARCIA, APRIL R</t>
+          <t>RODRIGUEZ, AGUSTIN</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1187 E 500 NORTH</t>
+          <t>2570 W PEBBLE CREEK LN</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1861,7 +1865,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>84043-1311</t>
+          <t>84043</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1873,22 +1877,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>GARCIA, ARMANDO</t>
+          <t>RODRIGUEZ, ALBERTO</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1457 N 460 WEST</t>
+          <t>4576 N BROWNING WAY</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PLEASANT GROVE</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>84062-3859</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -1900,22 +1904,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>GARCIA, ARMANDO CASTELAN</t>
+          <t>RODRIGUEZ, ALBERTO VAZQUEZ</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>4043 S LAKE MOUNTAIN DR</t>
+          <t>1525 W 300 NORTH</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>SARATOGA SPRINGS</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84062</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -1927,12 +1931,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>GARCIA, ARNULFO</t>
+          <t>RODRIGUEZ, ALEJANDRA</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>3718 N BOUNTIFUL LN</t>
+          <t>1771 E SKYLINE DR</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1954,22 +1958,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>GARCIA, ARTURO</t>
+          <t>RODRIGUEZ, ALEJANDRO</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>321 W 600 SOUTH</t>
+          <t>1505 N 150 EAST</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>PAYSON</t>
+          <t>SPRINGVILLE</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>84651-2827</t>
+          <t>84663-3156</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -1981,12 +1985,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>GARCIA, ARTURO</t>
+          <t>RODRIGUEZ, ALEJANDRO ERNESTO CEVALLOS</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>543 W 1260 NORTH</t>
+          <t>3684 W BIG HORN DR</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1996,7 +2000,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>95242</t>
+          <t>84043</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2008,22 +2012,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>GARCIA, ARTURO SR</t>
+          <t>RODRIGUEZ, ALEX PRADO</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>1017 W 550 NORTH</t>
+          <t>7782 N SADDLEBACK DR</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>PLEASANT GROVE</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>84062-2175</t>
+          <t>84005-4486</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2035,12 +2039,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GARCIA, AUSTREBERTO</t>
+          <t>RODRIGUEZ, ALEXIS</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>348 S 2430 WEST</t>
+          <t>1198 S 1220 WEST</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2050,7 +2054,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>84601-3696</t>
+          <t>84601</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2062,22 +2066,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>GARCIA, AZGAD BANI</t>
+          <t>MARTINEZ FAMILY LIVING TRUST 12-17-2021</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>1018 W 1620 SOUTH</t>
+          <t>3077 S WILLOW CREEK DR</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>PAYSON</t>
+          <t>SARATOGA SPRINGS</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>84651</t>
+          <t>84045</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2089,24 +2093,20 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>GARCIA, BENITO ALFONSO JUAREZ</t>
+          <t>MARTINEZ FAMILY TRUST 04-23-2020 THE</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>1191 E BELL BUOY WAY</t>
+          <t>39 W HOLLYHOCK CIR</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>84005</t>
-        </is>
-      </c>
+          <t>SARATOGA SPRINGS</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>Owner</t>
@@ -2116,22 +2116,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>GARCIA, BERENICE</t>
+          <t>MARTINEZ FAMILY TRUST 11-25-2020 THE</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>962 E 40 NORTH</t>
+          <t>3409 N 750 EAST</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>LEHI</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>84663-1630</t>
+          <t>84043</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2143,22 +2143,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>GARCIA, BERENICE</t>
+          <t>MARTINEZ LEON, RODRIGO A</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>1494 N 1200 WEST</t>
+          <t>407 N PEACH ST</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>SANTAQUIN</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>84057-2450</t>
+          <t>84655-8282</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2170,22 +2170,14 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>GARCIA, BETSY P</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>1495 W 200 SOUTH</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>LEHI</t>
-        </is>
-      </c>
+          <t>MARTINEZ LEON, RODRIGO A</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>84043-3684</t>
+          <t>84655-8282</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2197,22 +2189,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GARCIA, BETTY L</t>
+          <t>MARTINEZ LIVING TRUST 06-16-2025 THE</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>97 N 1100 EAST</t>
+          <t>1765 N 1450 WEST</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>AMERICAN FORK</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>84003-2917</t>
+          <t>90712</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2224,22 +2216,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>GARCIA, BLANCA E</t>
+          <t>MARTINEZ, ABEL E</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>1093 N 50 EAST</t>
+          <t>238 N 3000 WEST</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>84057-3237</t>
+          <t>84601-4022</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2251,22 +2243,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GARCIA, BLANCA ESMERALDA GUZMAN</t>
+          <t>MARTINEZ, ABEL IGNACIO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2254 W 1750 NORTH</t>
+          <t>1190 W PATCHWORK DR</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>LEHI</t>
+          <t>SANTAQUIN</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>84043-3214</t>
+          <t>84655</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2278,22 +2270,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>GARCIA, BONNIE</t>
+          <t>MARTINEZ, ADA L</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2832 S DRAKE AVE</t>
+          <t>2871 W 1100 NORTH</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SARATOGA SPRINGS</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84601-1735</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2305,22 +2297,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>GARCIA, BRANDEN CHRISTOPHER FLORES</t>
+          <t>MARTINEZ, ADALBERTO</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>1698 E BISON DR</t>
+          <t>1203 E 500 SOUTH</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>SPANISH FORK</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84660-2603</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2332,22 +2324,22 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>GARCIA, BRIANNA</t>
+          <t>MARTINEZ, ADDISON LAURIE</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>229 W 100 NORTH</t>
+          <t>558 W 800 SOUTH</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>LEHI</t>
+          <t>SPRINGVILLE</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>84043-1726</t>
+          <t>80111</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2359,18 +2351,22 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>GARCIA, BRIANNA</t>
+          <t>MARTINEZ, ADELAYDO</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>LEHI</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr"/>
+          <t>17579 S TUNNEL RD</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ELBERTA</t>
+        </is>
+      </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>84043-1726</t>
+          <t>84626-0146</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2382,22 +2378,22 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>GARCIA, BRITTNIE D</t>
+          <t>MARTINEZ, ADRIANA</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>182 E 400 SOUTH</t>
+          <t>1887 N 3410 WEST</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>GENOLA</t>
+          <t>LEHI</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>84655</t>
+          <t>33156</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2409,22 +2405,22 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>GARCIA, BRYAN ARCOS</t>
+          <t>MARTINEZ, ADRIANA ABIGAIL</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>7216 N BROOK RDG</t>
+          <t>1918 W 1020 NORTH</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84604-6129</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2436,22 +2432,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>GARCIA, BRYN BOWEN</t>
+          <t>MARTINEZ, ADRIANA BORJAS</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>437 N 700 EAST</t>
+          <t>1544 N 1825 WEST</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>LEHI</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>84097-4293</t>
+          <t>84043-3674</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2463,22 +2459,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GARCIA, CAMILA A</t>
+          <t>MARTINEZ, AGUSTIN</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>1152 W HIDDEN SPRING DR</t>
+          <t>4526 E SILVER MOON DR</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>SANTAQUIN</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>84655</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -2490,22 +2486,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>GARCIA, CARINA M</t>
+          <t>MARTINEZ, AGUSTIN E GORDILLO</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>947 N SILVER WOLF RD</t>
+          <t>771 S 100 WEST</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ELK RIDGE</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>84651</t>
+          <t>84058-6285</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2517,22 +2513,22 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>GARCIA, CARLOS</t>
+          <t>MARTINEZ, AIMIE K</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>60 E GINGER GOLD RD</t>
+          <t>928 W PRAIRIE DOG WY</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SANTAQUIN</t>
+          <t>SARATOGA SPRINGS</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>84655</t>
+          <t>84045</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -2544,22 +2540,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>GARCIA, CARLOS</t>
+          <t>MARTINEZ, ALANNA</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>756 W 60 NORTH</t>
+          <t>3786 N BROWNING ST</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>SPANISH FORK</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>84660-2066</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -2571,22 +2567,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>GARCIA, CARLOS A</t>
+          <t>MARTINEZ, ALBERTO</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>550 N 800 EAST</t>
+          <t>235 W 300 NORTH</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>SANTAQUIN</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>84663-1121</t>
+          <t>84655-7041</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2598,22 +2594,22 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>GARCIA, CARLOS A</t>
+          <t>MARTINEZ, ALBERTO</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>934 E 880 NORTH</t>
+          <t>5132 E TAHOE WAY</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>84097-3444</t>
+          <t>84043</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -2625,22 +2621,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>GARCIA, CARLOS L</t>
+          <t>MARTINEZ, ALEC XAVIER MEJORADA</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>825 N 1120 EAST</t>
+          <t>3308 W 1570 NORTH</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>SPANISH FORK</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>84660</t>
+          <t>84601</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -2652,22 +2648,22 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GARCIA, CARLOS NAVARRO</t>
+          <t>MARTINEZ, ALEJANDRA</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>553 E 100 NORTH</t>
+          <t>99 E 700 SOUTH</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>PAYSON</t>
+          <t>LEHI</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>84651-2341</t>
+          <t>84043</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -2679,22 +2675,22 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GARCIA, CARLOS RODRIGUEZ</t>
+          <t>MARTINEZ, ALEJANDRO</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>4532 N MAPLE DR</t>
+          <t>1092 N STORY DR</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>LEHI</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84043</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -2706,22 +2702,22 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>GARCIA, CARMEN</t>
+          <t>MARTINEZ, ALFA L</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>1838 W WEMBLEY PARK</t>
+          <t>435 N 300 WEST</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>84663</t>
+          <t>84057-3867</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -2733,22 +2729,22 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>GARCIA, CAROLINA</t>
+          <t>MARTINEZ, ALFONSO A LUNA</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>1502 W 610 SOUTH</t>
+          <t>5073 E LAKEFIELD DR</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>84058-4986</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -2760,22 +2756,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GARCIA, CATALINA</t>
+          <t>MARTINEZ, ALFREDO</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>33 E 400 SOUTH</t>
+          <t>797 W 600 NORTH</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>PROVO</t>
+          <t>LINDON</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>84606-4664</t>
+          <t>84042</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -2787,12 +2783,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GARCIA, CELIA</t>
+          <t>MARTINEZ, ALLISON MORGAN</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>7216 N BROOK RDG</t>
+          <t>6216 N BOULTER PEAK LN</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2814,22 +2810,22 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GARCIA, CESAR D</t>
+          <t>MARTINEZ, ALMA R REYES</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>296 W 1800 SOUTH</t>
+          <t>255 E 1230 NORTH</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>PAYSON</t>
+          <t>SPRINGVILLE</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>84651</t>
+          <t>84663-1131</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -2841,22 +2837,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>GARCIA, CESAR E</t>
+          <t>MARTINEZ, ALYSSA C</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>224 E EVERGREEN RD</t>
+          <t>135 W 400 SOUTH</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>AMERICAN FORK</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>84663-9458</t>
+          <t>84003-2652</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -2868,12 +2864,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GARCIA, CESAR GONZALEZ</t>
+          <t>HERNANDEZ CARBAJAL, JUAN C</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>280 W 205 NORTH</t>
+          <t>1140 W 950 NORTH</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2883,7 +2879,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>84057-4681</t>
+          <t>84057</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -2895,22 +2891,22 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>GARCIA, CESAR JAVIER</t>
+          <t>HERNANDEZ FAMILY 2011 REVOCABLE TRUST 11-09-2011</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>475 W 1890 SOUTH</t>
+          <t>15324 S LAKE BLUFF DR</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>PAYSON</t>
+          <t>DRAPER</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>84651</t>
+          <t>84020</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -2922,12 +2918,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>GARCIA, CESAR VALADEZ</t>
+          <t>HERNANDEZ FAMILY REVOCABLE LIVING TRUST 06-14-2019 THE</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>1451 S 240 EAST</t>
+          <t>362 N 900 EAST</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2937,7 +2933,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>84058-7607</t>
+          <t>84097-5043</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -2949,22 +2945,22 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>GARCIA, CHANDLER</t>
+          <t>HERNANDEZ FAMILY TRUST 06-25-2025 THE</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>1038 W 980 SOUTH</t>
+          <t>848 N 500 EAST</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>AMERICAN FORK</t>
+          <t>SPRINGVILLE</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>84003</t>
+          <t>84663-1481</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -2976,22 +2972,22 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>GARCIA, CHELSEA</t>
+          <t>HERNANDEZ FAMILY TRUST 10-14-2021</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>339 STONE DR</t>
+          <t>2313 W 490 SOUTH CIR</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>SANTAQUIN</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>84655</t>
+          <t>84601</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -3003,22 +2999,22 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>GARCIA, CHELSEA MARIE</t>
+          <t>HERNANDEZ FLORES, MA DEL REFUGIO</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>1241 E PAMELA ST</t>
+          <t>1540 S 175 EAST</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84058-7694</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -3030,12 +3026,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>GARCIA, CHRIS</t>
+          <t>HERNANDEZ FLORES, MA DEL REFUGIO</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>79 N 380 WEST</t>
+          <t>1533 S 125 EAST</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3045,7 +3041,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>84057-4628</t>
+          <t>84058-7677</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -3057,22 +3053,22 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>GARCIA, CHRISTIAN</t>
+          <t>HERNANDEZ FLORES, MA DEL REFUGIO</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>364 S 1000 WEST</t>
+          <t>1140 W 950 NORTH</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>PAYSON</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>84651-2451</t>
+          <t>84057</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -3084,22 +3080,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>GARCIA, CHRISTIAN</t>
+          <t>HERNANDEZ LIVING TRUST 03-31-2022</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>3326 E CALEDONIA AVE</t>
+          <t>108 W 400 NORTH</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>AMERICAN FORK</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>90630</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -3111,22 +3107,22 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>GARCIA, CHRISTIAN ANDRES CANTOR</t>
+          <t>HERNANDEZ, AARON</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>1219 N CHRISTLEY LN</t>
+          <t>492 E APPLE BLOSSOM LN</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ELK RIDGE</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>84651</t>
+          <t>84062</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -3138,22 +3134,22 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>GARCIA, CHRISTINE</t>
+          <t>HERNANDEZ, AARON MALPICA</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>1045 S 1700 WEST BLDG 2</t>
+          <t>1700 S SANDHILL RD</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>PAYSON</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>84651</t>
+          <t>84058</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -3165,22 +3161,22 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>GARCIA, CHRISTOPHER</t>
+          <t>HERNANDEZ, ABRAHAM</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>989 W 1000 SOUTH</t>
+          <t>1016 S 2480 EAST</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>SPANISH FORK</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>84663-5525</t>
+          <t>84660-3510</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -3192,12 +3188,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>GARCIA, CHRISTOPHER ALLEN</t>
+          <t>HERNANDEZ, ADRIANA INIGUEZ</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>1921 E 900 NORTH</t>
+          <t>1462 N SUNSET DR</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3219,12 +3215,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>GARCIA, CHRISTOPHER IRVIN</t>
+          <t>HERNANDEZ, ADRIANA MORENO</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>509 N EMERY AVE</t>
+          <t>708 E 1700 SOUTH</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3234,7 +3230,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>84057</t>
+          <t>84097-8023</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -3246,22 +3242,22 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>GARCIA, CHRISTOPHER MARTIN</t>
+          <t>HERNANDEZ, ADRIANA VANESSA COSTA</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>1296 S SAGEHILL DR</t>
+          <t>818 W 1100 NORTH</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>SANTAQUIN</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>84655</t>
+          <t>84062-9646</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -3273,22 +3269,22 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>GARCIA, CINDY E</t>
+          <t>HERNANDEZ, AIONA</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>557 W DEVON GLEN DR</t>
+          <t>14869 S VILLAGE CREST DR</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>DRAPER</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>84663</t>
+          <t>84020</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -3300,22 +3296,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>GARCIA, CINTHYA CISNEROS</t>
+          <t>HERNANDEZ, ALBERTO</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2111 E EAGLE CREST WY</t>
+          <t>913 S ARTESIAN RD</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84058</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -3327,22 +3323,22 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>GARCIA, CLAUDIA</t>
+          <t>HERNANDEZ, ALBERTO</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>25 W HALE DR</t>
+          <t>7212 N HIDDEN STEPPE BND</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>PLEASANT GROVE</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>84062</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -3354,22 +3350,22 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>GARCIA, CLAUDIA</t>
+          <t>HERNANDEZ, ALEJANDRA</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>3039 E 80 SOUTH</t>
+          <t>1212 W SPENCER RD</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>SPANISH FORK</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>84660</t>
+          <t>84062</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -3381,22 +3377,22 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>GARCIA, CLAUDIA E</t>
+          <t>HERNANDEZ, ALEX</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>1754 N KILLDEER DR</t>
+          <t>1386 E 410 SOUTH</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>SALEM</t>
+          <t>SPANISH FORK</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>84653</t>
+          <t>84660-2375</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -3408,22 +3404,22 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>GARCIA, CLAUDIA ESTEVES</t>
+          <t>HERNANDEZ, ALEXANDER</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>1766 W 80 SOUTH</t>
+          <t>72 W 750 NORTH</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>PROVO</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>84601-3803</t>
+          <t>84057-3834</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -3435,22 +3431,22 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GARCIA, CLAUDIA S CORRAL</t>
+          <t>HERNANDEZ, ALEXANDER J HERNANDEZ</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>1648 E 950 SOUTH</t>
+          <t>706 N BOSEMAN WAY</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>SPANISH FORK</t>
+          <t>SARATOGA SPRINGS</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>84660-9410</t>
+          <t>84045</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -3462,22 +3458,22 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GARCIA, CLAUDIA SANDOVAL</t>
+          <t>HERNANDEZ, ALEXANDRA</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>716 S 1400 WEST</t>
+          <t>9307 N TAMPA DR</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>PROVO</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>84601</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -3489,22 +3485,22 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>GARCIA, CLAUDIA SARAHI CORRAL</t>
+          <t>HERNANDEZ, ALFREDO J RODRIGUEZ</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>251 S 1000 EAST</t>
+          <t>3773 N CUADE ST</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>PROVO</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>84660-9410</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -3516,22 +3512,22 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>GARCIA, CLIFF MATTHEW</t>
+          <t>HERNANDEZ, ALFREDO Z</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>1751 N 3830 WEST</t>
+          <t>371 S 1000 WEST</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>LEHI</t>
+          <t>PAYSON</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>84043</t>
+          <t>84651-2450</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -3543,22 +3539,22 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>GARCIA, CONSUELO</t>
+          <t>HERNANDEZ, ALICEA</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>1159 N 800 WEST</t>
+          <t>736 N 390 EAST</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>AMERICAN FORK</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>84057-3031</t>
+          <t>84003-1371</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -3570,12 +3566,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>GARCIA, CORINNE</t>
+          <t>HERNANDEZ, ANA D ARIAS</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>1883 N BOUNTIFUL WY</t>
+          <t>863 N COULSEN DR</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3597,22 +3593,22 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>GARCIA, CRISTINA</t>
+          <t>HERNANDEZ, ANA MARIA</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>670 N ATLANTIS DR</t>
+          <t>895 N 400 EAST</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>84057-4038</t>
+          <t>84062-1803</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -3624,22 +3620,22 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>GARCIA, CRUZ F</t>
+          <t>HERNANDEZ, ANA MARIA PULIDO</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>216 S 540 EAST</t>
+          <t>894 N 1330 EAST</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>LEHI</t>
+          <t>SPANISH FORK</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>84043-2272</t>
+          <t>84660</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -3651,22 +3647,22 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>GARCIA, CRYSTAL YUKINO HOKANSON</t>
+          <t>HERNANDEZ, ANGEL</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>1096 E DORY BOAT RD</t>
+          <t>1315 N 2770 WEST</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>SARATOGA SPRINGS</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84601-1193</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -3678,22 +3674,22 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>GARCIA, DANIA</t>
+          <t>LOPEZ 9086 LLC</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>428 W 645 SOUTH</t>
+          <t>9086 N SILVER LAKE DR</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>FAIRFIELD</t>
+          <t>CEDAR HILLS</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84062-8787</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -3705,18 +3701,22 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>GARCIA, DANIA SANDOVAL</t>
+          <t>LOPEZ FAMILY TRUST 09-24-2019 THE</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>SARATOGA SPRINGS</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr"/>
+          <t>397 N CHERRY LN</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>SANTAQUIN</t>
+        </is>
+      </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84655</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -3728,22 +3728,22 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>GARCIA, DANIA SANDOVAL</t>
+          <t>LOPEZ, ABEL URIBE</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>3948 S PANORAMA DR</t>
+          <t>510 S TURLEY AVE</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>SARATOGA SPRINGS</t>
+          <t>PLEASANT GROVE</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84601-5500</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -3755,24 +3755,20 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>GARCIA, DANIEL</t>
+          <t>LOPEZ, ABISH GABRIELA</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>139 E 1200 NORTH</t>
+          <t>1173 S SLATE CANYON DR</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>OREM</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>84057-2707</t>
-        </is>
-      </c>
+          <t>PROVO</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
           <t>Owner</t>
@@ -3782,22 +3778,22 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>GARCIA, DANIEL AARON MARTINEZ</t>
+          <t>LOPEZ, ABRAHAM CARRASCO</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2041 E CANYONLANDS LN</t>
+          <t>456 W 1890 SOUTH</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>PAYSON</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84651</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -3809,22 +3805,22 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>GARCIA, DANIEL ARCOS</t>
+          <t>LOPEZ, ABRIL</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>1398 N 80 WEST</t>
+          <t>524 N 2870 WEST</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>84057-8325</t>
+          <t>84601-8264</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -3836,22 +3832,22 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>GARCIA, DANIEL BRANDON</t>
+          <t>LOPEZ, ADALBERTO</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>939 W LITTLE TIGER CT</t>
+          <t>1815 S 825 WEST</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>SARATOGA SPRINGS</t>
+          <t>LEHI</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84043-5475</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -3863,22 +3859,22 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>GARCIA, DANIEL E</t>
+          <t>LOPEZ, ADRIANA B VERGARAY</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>364 W 650 NORTH</t>
+          <t>1806 W 1120 SOUTH</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>SANTAQUIN</t>
+          <t>SPRINGVILLE</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>84655-5109</t>
+          <t>84047</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -3890,22 +3886,22 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>GARCIA, DANIEL LEIGH</t>
+          <t>LOPEZ, ADRIANA MARIA OLIVERA</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>9881 N CAMBRIDGE CT</t>
+          <t>519 W 530 SOUTH</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>HIGHLAND</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>84003-3461</t>
+          <t>84058-6123</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -3917,22 +3913,22 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>GARCIA, DANIEL SANCHEZ</t>
+          <t>LOPEZ, AGUSTIN F SANCHEZ</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>87 N KINTAIL ST</t>
+          <t>1081 S 680 WEST</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>SARATOGA SPRINGS</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84601-5558</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -3944,22 +3940,22 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>GARCIA, DANIELA JIMENEZ</t>
+          <t>LOPEZ, AGUSTINE LEONARDO IV</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>846 N 300 WEST</t>
+          <t>3707 N SUMMER WAY</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>LEHI</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>84043-1523</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -3971,22 +3967,22 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>GARCIA, DANIELLE</t>
+          <t>LOPEZ, AIDA SAMAYOA</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>3326 E CALEDONIA AVE</t>
+          <t>1048 E RIVERSIDE LN</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84097</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -3998,22 +3994,22 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>GARCIA, DAVID</t>
+          <t>LOPEZ, ALBA L</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>487 W 200 SOUTH</t>
+          <t>1404 N 800 WEST</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>84663-4906</t>
+          <t>84057-2964</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -4025,22 +4021,22 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>GARCIA, DAVID</t>
+          <t>LOPEZ, ALBERTO HERNANDEZ</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>10034 N MARIGOLD LN</t>
+          <t>1122 W 600 SOUTH</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>CEDAR HILLS</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>84660-2977</t>
+          <t>84058-5933</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -4052,14 +4048,22 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>GARCIA, DAVID GARCIA</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr"/>
-      <c r="C136" t="inlineStr"/>
+          <t>LOPEZ, ALBERTO JUAREZ</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>569 E STONEBRIAR DR</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>EAGLE MOUNTAIN</t>
+        </is>
+      </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>84660</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -4071,22 +4075,22 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>GARCIA, DAVID GARCIA</t>
+          <t>LOPEZ, ALDO GABRIEL</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2295 W 610 SOUTH</t>
+          <t>2326 W 490 SOUTH CIR</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>PLEASANT GROVE</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>84062</t>
+          <t>84601</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -4098,22 +4102,22 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>GARCIA, DAVID GARCIA</t>
+          <t>LOPEZ, ALEJANDRA</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>830 E SCENIC DR</t>
+          <t>696 S 1040 WEST</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>SPANISH FORK</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>84660</t>
+          <t>84058-5905</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -4125,22 +4129,22 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>GARCIA, DAYANA AGUERO</t>
+          <t>LOPEZ, ALEJANDRA MORENO</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>841 W FALLOW DR</t>
+          <t>1281 S 3500 EAST</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>SARATOGA SPRINGS</t>
+          <t>SPANISH FORK</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84660</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -4152,22 +4156,22 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>GARCIA, DEIRA ZAVALA</t>
+          <t>LOPEZ, ALEXANDRA DIAZ</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>221 S 1050 WEST</t>
+          <t>518 S 750 WEST</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>PROVO</t>
+          <t>SPANISH FORK</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>84601</t>
+          <t>84660-5763</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -4179,22 +4183,22 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>GARCIA, DIANA</t>
+          <t>LOPEZ, ALFONZO ZAMORA</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>920 W 1340 NORTH</t>
+          <t>467 N 400 WEST</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>SANTAQUIN</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>84057</t>
+          <t>84655-7175</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -4206,12 +4210,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>GARCIA, DIANA RAMIREZ</t>
+          <t>LOPEZ, ALFREDO</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>341 W 200 NORTH</t>
+          <t>2511 W 710 NORTH</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -4221,7 +4225,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>84601-2759</t>
+          <t>84601-1141</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -4233,14 +4237,22 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>GARCIA, DIANE</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr"/>
-      <c r="C143" t="inlineStr"/>
+          <t>LOPEZ, ALFREDO NAVA</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>642 W 1000 SOUTH</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>SPRINGVILLE</t>
+        </is>
+      </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>84660-3501</t>
+          <t>84663</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -4252,14 +4264,22 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>GARCIA, DIANE</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr"/>
-      <c r="C144" t="inlineStr"/>
+          <t>LOPEZ, ALICIA</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>386 E DELANO PEAK RD</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>EAGLE MOUNTAIN</t>
+        </is>
+      </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>84660-3501</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -4271,22 +4291,22 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>GARCIA, DIANE</t>
+          <t>LOPEZ, ALICIA MIGUEL</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>836 S 1520 EAST</t>
+          <t>54 N NORTHSHORE DR</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>SPANISH FORK</t>
+          <t>SARATOGA SPRINGS</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>84660-3501</t>
+          <t>84045</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -4298,22 +4318,22 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>GARCIA, DIANNE</t>
+          <t>LOPEZ, ALISON</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>355 S 430 EAST</t>
+          <t>1732 E 850 NORTH</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>LEHI</t>
+          <t>SALEM</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>84043-2269</t>
+          <t>84653</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -4325,22 +4345,22 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>GARCIA, DIEGO ESTEBAN</t>
+          <t>LOPEZ, ALLAN</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>798 N 250 WEST</t>
+          <t>3579 E ROCK CREEK RD</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>SPRINGVILLE</t>
+          <t>EAGLE MOUNTAIN</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>84663-1267</t>
+          <t>84005</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -4352,22 +4372,22 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>GARCIA, DIEGO MORALES</t>
+          <t>LOPEZ, ALMA D</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>449 W 1950 NORTH</t>
+          <t>1393 W 1350 SOUTH</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>OREM</t>
+          <t>SPRINGVILLE</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>84057</t>
+          <t>84663-3550</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -4379,22 +4399,22 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>GARCIA, DIEGO O</t>
+          <t>LOPEZ, ALMA R</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>3122 E QUAIL CT</t>
+          <t>693 W 1450 SOUTH</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>EAGLE MOUNTAIN</t>
+          <t>SPRINGVILLE</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>84005</t>
+          <t>84663</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -4406,22 +4426,22 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>GARCIA, E JOSEFINA</t>
+          <t>LOPEZ, ALMA T</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>199 S 1860 WEST</t>
+          <t>671 W 640 NORTH</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>PROVO</t>
+          <t>OREM</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>84601-3857</t>
+          <t>84057-3613</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -4433,22 +4453,22 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>GARCIA, EDEN RAMONA IZARRA</t>
+          <t>LOPEZ, ALONDRA W</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>881 N COULSEN DR</t>
+          <t>943 W 1500 SOUTH</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>SARATOGA SPRINGS</t>
+          <t>PROVO</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>84045</t>
+          <t>84601-5550</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">

</xml_diff>